<commit_message>
feat: add CW# keyword; post-generation missing-fields summary popup
</commit_message>
<xml_diff>
--- a/data/settlement info/settlement info.xlsx
+++ b/data/settlement info/settlement info.xlsx
@@ -5,16 +5,19 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\LiMa595\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://hp.sharepoint.com/teams/InputDevice/Shared Documents/General/17. Automation Projects/settlement-form-generator/data/settlement info/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EFC9C18D-6AB1-419E-98A5-91AC95941D19}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="10" documentId="13_ncr:1_{EFC9C18D-6AB1-419E-98A5-91AC95941D19}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D7C4DD2E-A380-4740-8E99-C07E8E7D3721}"/>
   <bookViews>
-    <workbookView xWindow="260" yWindow="1110" windowWidth="17460" windowHeight="9730" xr2:uid="{B4B4C7C1-7052-47F5-B23D-E78807A6AB18}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{B4B4C7C1-7052-47F5-B23D-E78807A6AB18}"/>
   </bookViews>
   <sheets>
     <sheet name="Supplier Info" sheetId="1" r:id="rId1"/>
   </sheets>
+  <externalReferences>
+    <externalReference r:id="rId2"/>
+  </externalReferences>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -39,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="228" uniqueCount="134">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="229" uniqueCount="135">
   <si>
     <t>GBU</t>
   </si>
@@ -335,12 +338,6 @@
     <t>LITE-ON TECHNOLOGY CORPORATION</t>
   </si>
   <si>
-    <t>Jerry Hsu</t>
-  </si>
-  <si>
-    <t>IT&amp;CE SBG Head</t>
-  </si>
-  <si>
     <t>SR_000029</t>
   </si>
   <si>
@@ -441,6 +438,15 @@
   </si>
   <si>
     <t>ICMSRAgreementEffectiveDate</t>
+  </si>
+  <si>
+    <t>CW#</t>
+  </si>
+  <si>
+    <t>Anson Chiu</t>
+  </si>
+  <si>
+    <t>President</t>
   </si>
 </sst>
 </file>
@@ -508,7 +514,10 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="2">
+  <dxfs count="3">
+    <dxf>
+      <numFmt numFmtId="164" formatCode="[$-409]mmmm\ d\,\ yyyy;@"/>
+    </dxf>
     <dxf>
       <numFmt numFmtId="164" formatCode="[$-409]mmmm\ d\,\ yyyy;@"/>
     </dxf>
@@ -547,10 +556,277 @@
 </styleSheet>
 </file>
 
+<file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
+  <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
+    <xxl21:alternateUrls>
+      <xxl21:absoluteUrl r:id="rId2"/>
+      <xxl21:relativeUrl r:id="rId3"/>
+    </xxl21:alternateUrls>
+    <sheetNames>
+      <sheetName val="Supplier Info"/>
+      <sheetName val="List"/>
+      <sheetName val="Data"/>
+    </sheetNames>
+    <sheetDataSet>
+      <sheetData sheetId="0">
+        <row r="1">
+          <cell r="D1" t="str">
+            <v>Supplier name</v>
+          </cell>
+          <cell r="E1" t="str">
+            <v>Master Agreement</v>
+          </cell>
+        </row>
+        <row r="2">
+          <cell r="D2" t="str">
+            <v>HOKG KONG JRD PRECISION MECHANICAL COMPANY LIMITED</v>
+          </cell>
+          <cell r="E2" t="str">
+            <v>CW2291673</v>
+          </cell>
+        </row>
+        <row r="3">
+          <cell r="D3" t="str">
+            <v>Bin Chuan Enterprise Co., LTD.</v>
+          </cell>
+          <cell r="E3" t="str">
+            <v>CW2291675</v>
+          </cell>
+        </row>
+        <row r="4">
+          <cell r="D4" t="str">
+            <v>Zhuchang Precision Optical Machinery (Shanghai) Co. Ltd.</v>
+          </cell>
+          <cell r="E4" t="str">
+            <v>CW2291677</v>
+          </cell>
+        </row>
+        <row r="5">
+          <cell r="D5" t="str">
+            <v>DYNAMIC APEX LIMITED</v>
+          </cell>
+          <cell r="E5" t="str">
+            <v>CW2291682</v>
+          </cell>
+        </row>
+        <row r="6">
+          <cell r="D6" t="str">
+            <v>KENSEISHA(SHANGHAI) PRECISION MACHINING PROCESS CO., LTD.</v>
+          </cell>
+          <cell r="E6" t="str">
+            <v>CW2291684</v>
+          </cell>
+        </row>
+        <row r="7">
+          <cell r="D7" t="str">
+            <v>Catcher Technology Co., Ltd</v>
+          </cell>
+          <cell r="E7" t="str">
+            <v>CW2291686</v>
+          </cell>
+        </row>
+        <row r="8">
+          <cell r="D8" t="str">
+            <v>KA SHUI MANUFACTORY CO., LTD</v>
+          </cell>
+          <cell r="E8" t="str">
+            <v>CW2291688</v>
+          </cell>
+        </row>
+        <row r="9">
+          <cell r="D9" t="str">
+            <v>CHONGQING BAI YU SHUN TECHNOLOGY COMPANY</v>
+          </cell>
+          <cell r="E9" t="str">
+            <v>CW2290251</v>
+          </cell>
+        </row>
+        <row r="10">
+          <cell r="D10" t="str">
+            <v>DONGGUAN SHANGZHUN HARDWARE CO LTD</v>
+          </cell>
+          <cell r="E10" t="str">
+            <v>CW2291690</v>
+          </cell>
+        </row>
+        <row r="11">
+          <cell r="D11" t="str">
+            <v>Kunshan Denghe precision Machinery Co.,Ltd</v>
+          </cell>
+          <cell r="E11" t="str">
+            <v>CW2291692</v>
+          </cell>
+        </row>
+        <row r="12">
+          <cell r="D12" t="str">
+            <v>MAANSHAN GREEN DESIGN ELECTRONICS TECHNOLOGY CO., LTD</v>
+          </cell>
+          <cell r="E12" t="str">
+            <v>CW2291694</v>
+          </cell>
+        </row>
+        <row r="13">
+          <cell r="D13" t="str">
+            <v>XINXIU Corporation</v>
+          </cell>
+          <cell r="E13" t="str">
+            <v>CW2291696</v>
+          </cell>
+        </row>
+        <row r="14">
+          <cell r="D14" t="str">
+            <v>CosmoSupplyLab</v>
+          </cell>
+          <cell r="E14" t="str">
+            <v>CW2291698</v>
+          </cell>
+        </row>
+        <row r="15">
+          <cell r="D15" t="str">
+            <v>LEONHARD KURZ Stiftung &amp; Co. KG</v>
+          </cell>
+          <cell r="E15" t="str">
+            <v>CW2291772</v>
+          </cell>
+        </row>
+        <row r="16">
+          <cell r="D16" t="str">
+            <v>SENTIEN PRINTING FACTORY CO., LTD.</v>
+          </cell>
+          <cell r="E16" t="str">
+            <v>CW2291700</v>
+          </cell>
+        </row>
+        <row r="17">
+          <cell r="D17" t="str">
+            <v>AURAS TECHNOLOGY CO., LTD</v>
+          </cell>
+          <cell r="E17" t="str">
+            <v>CW2291702</v>
+          </cell>
+        </row>
+        <row r="18">
+          <cell r="D18" t="str">
+            <v>SUNONWEALTH ELECTRIC MACHINE INDUSTRY CO., LTD</v>
+          </cell>
+          <cell r="E18" t="str">
+            <v>CW2291704</v>
+          </cell>
+        </row>
+        <row r="19">
+          <cell r="D19" t="str">
+            <v>DELTA ELECTRONICS INT’L (SINGAPORE) PTE. LTD</v>
+          </cell>
+          <cell r="E19" t="str">
+            <v>CW2291706</v>
+          </cell>
+        </row>
+        <row r="20">
+          <cell r="D20" t="str">
+            <v>Nidec Chaun-Choung Technology Corporation</v>
+          </cell>
+          <cell r="E20" t="str">
+            <v>CW2291708</v>
+          </cell>
+        </row>
+        <row r="21">
+          <cell r="D21" t="str">
+            <v>HUAYING ELECTRONICS TECHNOLOGY CO., LIMITED</v>
+          </cell>
+        </row>
+        <row r="22">
+          <cell r="D22" t="str">
+            <v>Asia Vital Components Co., Ltd.</v>
+          </cell>
+          <cell r="E22" t="str">
+            <v>CW2291710</v>
+          </cell>
+        </row>
+        <row r="23">
+          <cell r="D23" t="str">
+            <v xml:space="preserve">FORCECON TECHNOLOGY CO., LTD </v>
+          </cell>
+          <cell r="E23" t="str">
+            <v>CW2291712</v>
+          </cell>
+        </row>
+        <row r="24">
+          <cell r="D24" t="str">
+            <v>CHICONY ELECTRONICS CO., LTD.</v>
+          </cell>
+          <cell r="E24" t="str">
+            <v>CW2290757</v>
+          </cell>
+        </row>
+        <row r="25">
+          <cell r="D25" t="str">
+            <v>CHICONY ELECTRONICS CO., LTD.</v>
+          </cell>
+          <cell r="E25" t="str">
+            <v>CW2290757</v>
+          </cell>
+        </row>
+        <row r="26">
+          <cell r="D26" t="str">
+            <v>LITE-ON TECHNOLOGY CORPORATION</v>
+          </cell>
+          <cell r="E26" t="str">
+            <v>CW2290755</v>
+          </cell>
+        </row>
+        <row r="27">
+          <cell r="D27" t="str">
+            <v>PRIMAX ELECTRONICS LTD.</v>
+          </cell>
+          <cell r="E27" t="str">
+            <v>CW2290761</v>
+          </cell>
+        </row>
+        <row r="28">
+          <cell r="D28" t="str">
+            <v>DARFON ELECTRONICS CORP.</v>
+          </cell>
+          <cell r="E28" t="str">
+            <v>CW2290759</v>
+          </cell>
+        </row>
+        <row r="29">
+          <cell r="D29" t="str">
+            <v>SUNREX TECHNOLOGY CORP.</v>
+          </cell>
+          <cell r="E29" t="str">
+            <v>CW2290763</v>
+          </cell>
+        </row>
+        <row r="30">
+          <cell r="D30" t="str">
+            <v>ELAN MICROELECTRONICS CORPORATION</v>
+          </cell>
+          <cell r="E30" t="str">
+            <v>CW2290334</v>
+          </cell>
+        </row>
+        <row r="31">
+          <cell r="D31" t="str">
+            <v>Synaptics Incorporated</v>
+          </cell>
+          <cell r="E31" t="str">
+            <v>CW2290765</v>
+          </cell>
+        </row>
+      </sheetData>
+      <sheetData sheetId="1"/>
+      <sheetData sheetId="2"/>
+    </sheetDataSet>
+  </externalBook>
+</externalLink>
+</file>
+
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{3796E6C5-3477-484B-B58A-01ABDB0F987D}" name="Table1" displayName="Table1" ref="A1:J31" totalsRowShown="0" headerRowDxfId="1">
-  <autoFilter ref="A1:J31" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
-  <tableColumns count="10">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{3796E6C5-3477-484B-B58A-01ABDB0F987D}" name="Table1" displayName="Table1" ref="A1:K31" totalsRowShown="0" headerRowDxfId="2">
+  <autoFilter ref="A1:K31" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
+  <tableColumns count="11">
     <tableColumn id="1" xr3:uid="{8745379D-ABF7-4338-810D-020889C042C9}" name="Sub-Category"/>
     <tableColumn id="2" xr3:uid="{6495F64E-6439-4236-B965-B5AC3CA8DF4D}" name="GBU"/>
     <tableColumn id="3" xr3:uid="{BC823B95-0F4B-4DB1-A9E1-EC2D4D78D8FC}" name="GTK Supplier"/>
@@ -559,7 +835,10 @@
     <tableColumn id="8" xr3:uid="{5717F9AB-4028-41A3-8015-F5E1316E2840}" name="ICMExternalSignatoryTitle"/>
     <tableColumn id="5" xr3:uid="{B6AC2849-12D3-4ABE-8D3B-E69124505A5B}" name="ICMInternalSignatory"/>
     <tableColumn id="6" xr3:uid="{63B4BD2E-E735-483C-8AA0-A79412C44FA9}" name="ICMInternalSignatoryTitle"/>
-    <tableColumn id="9" xr3:uid="{13067000-AC71-4660-9DD9-E2AD30A83394}" name="ICMSRAgreementEffectiveDate" dataDxfId="0"/>
+    <tableColumn id="9" xr3:uid="{13067000-AC71-4660-9DD9-E2AD30A83394}" name="ICMSRAgreementEffectiveDate" dataDxfId="1"/>
+    <tableColumn id="11" xr3:uid="{EDA04414-F025-4CEE-AA09-0347A0AFF19A}" name="CW#" dataDxfId="0">
+      <calculatedColumnFormula>_xlfn.XLOOKUP(Table1[[#This Row],[ICMPartyName1]],'[1]Supplier Info'!$D:$D,'[1]Supplier Info'!$E:$E,,0)</calculatedColumnFormula>
+    </tableColumn>
     <tableColumn id="10" xr3:uid="{3309F73E-4CC4-4407-97D9-628068CBDF62}" name="ICMSRAGREEMENTCODE"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -883,7 +1162,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2BE11DAF-55AB-474F-9039-FABAB1A58A19}">
-  <dimension ref="A1:J31"/>
+  <dimension ref="A1:K31"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="18.08984375" customWidth="1"/>
@@ -892,42 +1171,46 @@
     <col min="4" max="4" width="58" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="19.1796875" customWidth="1"/>
     <col min="6" max="9" width="41.54296875" customWidth="1"/>
-    <col min="10" max="10" width="33.81640625" customWidth="1"/>
+    <col min="10" max="10" width="24.453125" customWidth="1"/>
+    <col min="11" max="11" width="33.81640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="D1" s="1" t="s">
+        <v>129</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>124</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>125</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>127</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>126</v>
+      </c>
+      <c r="I1" s="1" t="s">
         <v>131</v>
       </c>
-      <c r="E1" s="1" t="s">
-        <v>126</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>127</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>129</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>128</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>133</v>
-      </c>
       <c r="J1" s="1" t="s">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="2" spans="1:10" ht="16.5" customHeight="1" x14ac:dyDescent="0.35">
+        <v>132</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" ht="16.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>1</v>
       </c>
@@ -941,19 +1224,23 @@
         <v>4</v>
       </c>
       <c r="F2" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="G2" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="H2" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="I2" s="2">
         <v>45727</v>
       </c>
-    </row>
-    <row r="3" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="J2" s="2" t="str">
+        <f>_xlfn.XLOOKUP(Table1[[#This Row],[ICMPartyName1]],'[1]Supplier Info'!$D:$D,'[1]Supplier Info'!$E:$E,,0)</f>
+        <v>CW2291673</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>1</v>
       </c>
@@ -970,16 +1257,20 @@
         <v>9</v>
       </c>
       <c r="G3" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="H3" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="I3" s="2">
         <v>45722</v>
       </c>
-    </row>
-    <row r="4" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="J3" s="2" t="str">
+        <f>_xlfn.XLOOKUP(Table1[[#This Row],[ICMPartyName1]],'[1]Supplier Info'!$D:$D,'[1]Supplier Info'!$E:$E,,0)</f>
+        <v>CW2291675</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>1</v>
       </c>
@@ -996,16 +1287,20 @@
         <v>5</v>
       </c>
       <c r="G4" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="H4" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="I4" s="2">
         <v>45785</v>
       </c>
-    </row>
-    <row r="5" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="J4" s="2" t="str">
+        <f>_xlfn.XLOOKUP(Table1[[#This Row],[ICMPartyName1]],'[1]Supplier Info'!$D:$D,'[1]Supplier Info'!$E:$E,,0)</f>
+        <v>CW2291677</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>1</v>
       </c>
@@ -1022,16 +1317,20 @@
         <v>16</v>
       </c>
       <c r="G5" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="H5" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="I5" s="2">
         <v>45784</v>
       </c>
-    </row>
-    <row r="6" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="J5" s="2" t="str">
+        <f>_xlfn.XLOOKUP(Table1[[#This Row],[ICMPartyName1]],'[1]Supplier Info'!$D:$D,'[1]Supplier Info'!$E:$E,,0)</f>
+        <v>CW2291682</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>1</v>
       </c>
@@ -1048,16 +1347,20 @@
         <v>20</v>
       </c>
       <c r="G6" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="H6" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="I6" s="2">
         <v>45729</v>
       </c>
-    </row>
-    <row r="7" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="J6" s="2" t="str">
+        <f>_xlfn.XLOOKUP(Table1[[#This Row],[ICMPartyName1]],'[1]Supplier Info'!$D:$D,'[1]Supplier Info'!$E:$E,,0)</f>
+        <v>CW2291684</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>1</v>
       </c>
@@ -1074,16 +1377,20 @@
         <v>24</v>
       </c>
       <c r="G7" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="H7" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="I7" s="2">
         <v>45924</v>
       </c>
-    </row>
-    <row r="8" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="J7" s="2" t="str">
+        <f>_xlfn.XLOOKUP(Table1[[#This Row],[ICMPartyName1]],'[1]Supplier Info'!$D:$D,'[1]Supplier Info'!$E:$E,,0)</f>
+        <v>CW2291686</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>1</v>
       </c>
@@ -1100,16 +1407,20 @@
         <v>5</v>
       </c>
       <c r="G8" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="H8" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="I8" s="2">
         <v>45729</v>
       </c>
-    </row>
-    <row r="9" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="J8" s="2" t="str">
+        <f>_xlfn.XLOOKUP(Table1[[#This Row],[ICMPartyName1]],'[1]Supplier Info'!$D:$D,'[1]Supplier Info'!$E:$E,,0)</f>
+        <v>CW2291688</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>1</v>
       </c>
@@ -1126,16 +1437,20 @@
         <v>5</v>
       </c>
       <c r="G9" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="H9" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="I9" s="2">
         <v>45722</v>
       </c>
-    </row>
-    <row r="10" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="J9" s="2" t="str">
+        <f>_xlfn.XLOOKUP(Table1[[#This Row],[ICMPartyName1]],'[1]Supplier Info'!$D:$D,'[1]Supplier Info'!$E:$E,,0)</f>
+        <v>CW2290251</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>1</v>
       </c>
@@ -1152,16 +1467,20 @@
         <v>5</v>
       </c>
       <c r="G10" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="H10" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="I10" s="2">
         <v>45740</v>
       </c>
-    </row>
-    <row r="11" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="J10" s="2" t="str">
+        <f>_xlfn.XLOOKUP(Table1[[#This Row],[ICMPartyName1]],'[1]Supplier Info'!$D:$D,'[1]Supplier Info'!$E:$E,,0)</f>
+        <v>CW2291690</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>1</v>
       </c>
@@ -1178,16 +1497,20 @@
         <v>5</v>
       </c>
       <c r="G11" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="H11" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="I11" s="2">
         <v>45723</v>
       </c>
-    </row>
-    <row r="12" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="J11" s="2" t="str">
+        <f>_xlfn.XLOOKUP(Table1[[#This Row],[ICMPartyName1]],'[1]Supplier Info'!$D:$D,'[1]Supplier Info'!$E:$E,,0)</f>
+        <v>CW2291692</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>1</v>
       </c>
@@ -1204,16 +1527,20 @@
         <v>40</v>
       </c>
       <c r="G12" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="H12" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="I12" s="2">
         <v>45722</v>
       </c>
-    </row>
-    <row r="13" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="J12" s="2" t="str">
+        <f>_xlfn.XLOOKUP(Table1[[#This Row],[ICMPartyName1]],'[1]Supplier Info'!$D:$D,'[1]Supplier Info'!$E:$E,,0)</f>
+        <v>CW2291694</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>41</v>
       </c>
@@ -1230,14 +1557,18 @@
         <v>45</v>
       </c>
       <c r="G13" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="H13" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="I13" s="2"/>
-    </row>
-    <row r="14" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="J13" s="2" t="str">
+        <f>_xlfn.XLOOKUP(Table1[[#This Row],[ICMPartyName1]],'[1]Supplier Info'!$D:$D,'[1]Supplier Info'!$E:$E,,0)</f>
+        <v>CW2291696</v>
+      </c>
+    </row>
+    <row r="14" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>41</v>
       </c>
@@ -1254,16 +1585,20 @@
         <v>49</v>
       </c>
       <c r="G14" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="H14" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="I14" s="2">
         <v>45791</v>
       </c>
-    </row>
-    <row r="15" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="J14" s="2" t="str">
+        <f>_xlfn.XLOOKUP(Table1[[#This Row],[ICMPartyName1]],'[1]Supplier Info'!$D:$D,'[1]Supplier Info'!$E:$E,,0)</f>
+        <v>CW2291698</v>
+      </c>
+    </row>
+    <row r="15" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>50</v>
       </c>
@@ -1280,16 +1615,20 @@
         <v>54</v>
       </c>
       <c r="G15" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="H15" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="I15" s="2">
         <v>45740</v>
       </c>
-    </row>
-    <row r="16" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="J15" s="2" t="str">
+        <f>_xlfn.XLOOKUP(Table1[[#This Row],[ICMPartyName1]],'[1]Supplier Info'!$D:$D,'[1]Supplier Info'!$E:$E,,0)</f>
+        <v>CW2291772</v>
+      </c>
+    </row>
+    <row r="16" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>50</v>
       </c>
@@ -1306,16 +1645,20 @@
         <v>58</v>
       </c>
       <c r="G16" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="H16" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="I16" s="2">
         <v>45784</v>
       </c>
-    </row>
-    <row r="17" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="J16" s="2" t="str">
+        <f>_xlfn.XLOOKUP(Table1[[#This Row],[ICMPartyName1]],'[1]Supplier Info'!$D:$D,'[1]Supplier Info'!$E:$E,,0)</f>
+        <v>CW2291700</v>
+      </c>
+    </row>
+    <row r="17" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>59</v>
       </c>
@@ -1332,16 +1675,20 @@
         <v>63</v>
       </c>
       <c r="G17" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="H17" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="I17" s="2">
         <v>45740</v>
       </c>
-    </row>
-    <row r="18" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="J17" s="2" t="str">
+        <f>_xlfn.XLOOKUP(Table1[[#This Row],[ICMPartyName1]],'[1]Supplier Info'!$D:$D,'[1]Supplier Info'!$E:$E,,0)</f>
+        <v>CW2291702</v>
+      </c>
+    </row>
+    <row r="18" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>59</v>
       </c>
@@ -1358,14 +1705,18 @@
         <v>67</v>
       </c>
       <c r="G18" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="H18" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="I18" s="2"/>
-    </row>
-    <row r="19" spans="1:10" ht="16.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="J18" s="2" t="str">
+        <f>_xlfn.XLOOKUP(Table1[[#This Row],[ICMPartyName1]],'[1]Supplier Info'!$D:$D,'[1]Supplier Info'!$E:$E,,0)</f>
+        <v>CW2291704</v>
+      </c>
+    </row>
+    <row r="19" spans="1:11" ht="16.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>59</v>
       </c>
@@ -1382,14 +1733,18 @@
         <v>45</v>
       </c>
       <c r="G19" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="H19" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="I19" s="2"/>
-    </row>
-    <row r="20" spans="1:10" ht="16.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="J19" s="2" t="str">
+        <f>_xlfn.XLOOKUP(Table1[[#This Row],[ICMPartyName1]],'[1]Supplier Info'!$D:$D,'[1]Supplier Info'!$E:$E,,0)</f>
+        <v>CW2291706</v>
+      </c>
+    </row>
+    <row r="20" spans="1:11" ht="16.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>59</v>
       </c>
@@ -1406,16 +1761,20 @@
         <v>74</v>
       </c>
       <c r="G20" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="H20" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="I20" s="2">
         <v>45798</v>
       </c>
-    </row>
-    <row r="21" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="J20" s="2" t="str">
+        <f>_xlfn.XLOOKUP(Table1[[#This Row],[ICMPartyName1]],'[1]Supplier Info'!$D:$D,'[1]Supplier Info'!$E:$E,,0)</f>
+        <v>CW2291708</v>
+      </c>
+    </row>
+    <row r="21" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>59</v>
       </c>
@@ -1432,14 +1791,15 @@
         <v>78</v>
       </c>
       <c r="G21" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="H21" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="I21" s="2"/>
-    </row>
-    <row r="22" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="J21" s="2"/>
+    </row>
+    <row r="22" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>59</v>
       </c>
@@ -1456,14 +1816,18 @@
         <v>78</v>
       </c>
       <c r="G22" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="H22" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="I22" s="2"/>
-    </row>
-    <row r="23" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="J22" s="2" t="str">
+        <f>_xlfn.XLOOKUP(Table1[[#This Row],[ICMPartyName1]],'[1]Supplier Info'!$D:$D,'[1]Supplier Info'!$E:$E,,0)</f>
+        <v>CW2291710</v>
+      </c>
+    </row>
+    <row r="23" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>59</v>
       </c>
@@ -1480,14 +1844,18 @@
         <v>85</v>
       </c>
       <c r="G23" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="H23" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="I23" s="2"/>
-    </row>
-    <row r="24" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="J23" s="2" t="str">
+        <f>_xlfn.XLOOKUP(Table1[[#This Row],[ICMPartyName1]],'[1]Supplier Info'!$D:$D,'[1]Supplier Info'!$E:$E,,0)</f>
+        <v>CW2291712</v>
+      </c>
+    </row>
+    <row r="24" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
         <v>86</v>
       </c>
@@ -1507,19 +1875,23 @@
         <v>91</v>
       </c>
       <c r="G24" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="H24" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="I24" s="2">
         <v>45666</v>
       </c>
-      <c r="J24" t="s">
+      <c r="J24" s="2" t="str">
+        <f>_xlfn.XLOOKUP(Table1[[#This Row],[ICMPartyName1]],'[1]Supplier Info'!$D:$D,'[1]Supplier Info'!$E:$E,,0)</f>
+        <v>CW2290757</v>
+      </c>
+      <c r="K24" t="s">
         <v>92</v>
       </c>
     </row>
-    <row r="25" spans="1:10" ht="16.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:11" ht="16.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
         <v>86</v>
       </c>
@@ -1539,19 +1911,23 @@
         <v>95</v>
       </c>
       <c r="G25" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="H25" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="I25" s="2">
         <v>45666</v>
       </c>
-      <c r="J25" t="s">
+      <c r="J25" s="2" t="str">
+        <f>_xlfn.XLOOKUP(Table1[[#This Row],[ICMPartyName1]],'[1]Supplier Info'!$D:$D,'[1]Supplier Info'!$E:$E,,0)</f>
+        <v>CW2290757</v>
+      </c>
+      <c r="K25" t="s">
         <v>92</v>
       </c>
     </row>
-    <row r="26" spans="1:10" ht="16.5" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:11" ht="16.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
         <v>86</v>
       </c>
@@ -1562,160 +1938,184 @@
         <v>97</v>
       </c>
       <c r="E26" t="s">
-        <v>98</v>
+        <v>133</v>
       </c>
       <c r="F26" t="s">
-        <v>99</v>
+        <v>134</v>
       </c>
       <c r="G26" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="H26" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="I26" s="2">
         <v>45658</v>
       </c>
-      <c r="J26" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="27" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="J26" s="2" t="str">
+        <f>_xlfn.XLOOKUP(Table1[[#This Row],[ICMPartyName1]],'[1]Supplier Info'!$D:$D,'[1]Supplier Info'!$E:$E,,0)</f>
+        <v>CW2290755</v>
+      </c>
+      <c r="K26" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="27" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
         <v>86</v>
       </c>
       <c r="C27" t="s">
+        <v>99</v>
+      </c>
+      <c r="D27" t="s">
+        <v>100</v>
+      </c>
+      <c r="E27" t="s">
         <v>101</v>
       </c>
-      <c r="D27" t="s">
+      <c r="F27" t="s">
         <v>102</v>
       </c>
-      <c r="E27" t="s">
-        <v>103</v>
-      </c>
-      <c r="F27" t="s">
-        <v>104</v>
-      </c>
       <c r="G27" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="H27" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="I27" s="2">
         <v>45693</v>
       </c>
-      <c r="J27" t="s">
-        <v>105</v>
-      </c>
-    </row>
-    <row r="28" spans="1:10" ht="16.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="J27" s="2" t="str">
+        <f>_xlfn.XLOOKUP(Table1[[#This Row],[ICMPartyName1]],'[1]Supplier Info'!$D:$D,'[1]Supplier Info'!$E:$E,,0)</f>
+        <v>CW2290761</v>
+      </c>
+      <c r="K27" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="28" spans="1:11" ht="16.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
         <v>86</v>
       </c>
       <c r="C28" t="s">
+        <v>104</v>
+      </c>
+      <c r="D28" t="s">
+        <v>105</v>
+      </c>
+      <c r="E28" t="s">
         <v>106</v>
-      </c>
-      <c r="D28" t="s">
-        <v>107</v>
-      </c>
-      <c r="E28" t="s">
-        <v>108</v>
       </c>
       <c r="F28" t="s">
         <v>78</v>
       </c>
       <c r="G28" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="H28" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="I28" s="2">
         <v>45666</v>
       </c>
-      <c r="J28" t="s">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="29" spans="1:10" ht="16.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="J28" s="2" t="str">
+        <f>_xlfn.XLOOKUP(Table1[[#This Row],[ICMPartyName1]],'[1]Supplier Info'!$D:$D,'[1]Supplier Info'!$E:$E,,0)</f>
+        <v>CW2290759</v>
+      </c>
+      <c r="K28" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="29" spans="1:11" ht="16.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
         <v>86</v>
       </c>
       <c r="C29" t="s">
+        <v>108</v>
+      </c>
+      <c r="D29" t="s">
+        <v>109</v>
+      </c>
+      <c r="E29" t="s">
         <v>110</v>
-      </c>
-      <c r="D29" t="s">
-        <v>111</v>
-      </c>
-      <c r="E29" t="s">
-        <v>112</v>
       </c>
       <c r="F29" t="s">
         <v>63</v>
       </c>
       <c r="G29" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="H29" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="I29" s="2">
         <v>45672</v>
       </c>
-      <c r="J29" t="s">
+      <c r="J29" s="2" t="str">
+        <f>_xlfn.XLOOKUP(Table1[[#This Row],[ICMPartyName1]],'[1]Supplier Info'!$D:$D,'[1]Supplier Info'!$E:$E,,0)</f>
+        <v>CW2290763</v>
+      </c>
+      <c r="K29" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="30" spans="1:11" ht="16.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A30" t="s">
+        <v>112</v>
+      </c>
+      <c r="C30" t="s">
         <v>113</v>
       </c>
-    </row>
-    <row r="30" spans="1:10" ht="16.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A30" t="s">
+      <c r="D30" t="s">
         <v>114</v>
       </c>
-      <c r="C30" t="s">
+      <c r="E30" t="s">
         <v>115</v>
       </c>
-      <c r="D30" t="s">
+      <c r="F30" t="s">
         <v>116</v>
       </c>
-      <c r="E30" t="s">
-        <v>117</v>
-      </c>
-      <c r="F30" t="s">
-        <v>118</v>
-      </c>
       <c r="G30" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="H30" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="I30" s="2">
         <v>45714</v>
       </c>
-    </row>
-    <row r="31" spans="1:10" ht="16.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="J30" s="2" t="str">
+        <f>_xlfn.XLOOKUP(Table1[[#This Row],[ICMPartyName1]],'[1]Supplier Info'!$D:$D,'[1]Supplier Info'!$E:$E,,0)</f>
+        <v>CW2290334</v>
+      </c>
+    </row>
+    <row r="31" spans="1:11" ht="16.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="C31" t="s">
+        <v>117</v>
+      </c>
+      <c r="D31" t="s">
+        <v>118</v>
+      </c>
+      <c r="E31" t="s">
         <v>119</v>
-      </c>
-      <c r="D31" t="s">
-        <v>120</v>
-      </c>
-      <c r="E31" t="s">
-        <v>121</v>
       </c>
       <c r="F31" t="s">
         <v>5</v>
       </c>
       <c r="G31" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="H31" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="I31" s="2"/>
+      <c r="J31" s="2" t="str">
+        <f>_xlfn.XLOOKUP(Table1[[#This Row],[ICMPartyName1]],'[1]Supplier Info'!$D:$D,'[1]Supplier Info'!$E:$E,,0)</f>
+        <v>CW2290765</v>
+      </c>
     </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
@@ -1977,13 +2377,39 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{712A39FB-A1FD-418D-A657-32ECBACC94FF}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{712A39FB-A1FD-418D-A657-32ECBACC94FF}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="3ddbdfa1-be50-4b7a-b66f-14c4748c8596"/>
+    <ds:schemaRef ds:uri="2df2684a-2237-489e-8795-1f946593e18f"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{29D94F07-D8B4-4F0F-9836-65B41DA39758}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{29D94F07-D8B4-4F0F-9836-65B41DA39758}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1F55CD33-1A0B-42F8-BD7E-0D32351F432C}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1F55CD33-1A0B-42F8-BD7E-0D32351F432C}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="2df2684a-2237-489e-8795-1f946593e18f"/>
+    <ds:schemaRef ds:uri="3ddbdfa1-be50-4b7a-b66f-14c4748c8596"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
update settlement info; bump version to 0.3.2
</commit_message>
<xml_diff>
--- a/data/settlement info/settlement info.xlsx
+++ b/data/settlement info/settlement info.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://hp.sharepoint.com/teams/InputDevice/Shared Documents/General/17. Automation Projects/settlement-form-generator/data/settlement info/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="25" documentId="13_ncr:1_{EFC9C18D-6AB1-419E-98A5-91AC95941D19}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3763621B-2933-4A97-ABE1-BE7EA031BBCC}"/>
+  <xr:revisionPtr revIDLastSave="28" documentId="13_ncr:1_{EFC9C18D-6AB1-419E-98A5-91AC95941D19}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1858AAC7-D250-40AF-91D2-BC06E6EAAEF8}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{B4B4C7C1-7052-47F5-B23D-E78807A6AB18}"/>
   </bookViews>
@@ -1825,7 +1825,7 @@
         <v>121</v>
       </c>
       <c r="I26" s="2">
-        <v>45658</v>
+        <v>45670</v>
       </c>
       <c r="J26" s="2" t="s">
         <v>156</v>
@@ -1997,26 +1997,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="2df2684a-2237-489e-8795-1f946593e18f" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="3ddbdfa1-be50-4b7a-b66f-14c4748c8596">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100C7BB62D9C7AC4249BB50D4F119F8FF50" ma:contentTypeVersion="14" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="dab14850594d04436880d3464ba468af">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="3ddbdfa1-be50-4b7a-b66f-14c4748c8596" xmlns:ns3="2df2684a-2237-489e-8795-1f946593e18f" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="eb8d2f689c1774a9065a5e99593f72e7" ns2:_="" ns3:_="">
     <xsd:import namespace="3ddbdfa1-be50-4b7a-b66f-14c4748c8596"/>
@@ -2245,26 +2225,27 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1F55CD33-1A0B-42F8-BD7E-0D32351F432C}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="2df2684a-2237-489e-8795-1f946593e18f"/>
-    <ds:schemaRef ds:uri="3ddbdfa1-be50-4b7a-b66f-14c4748c8596"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{29D94F07-D8B4-4F0F-9836-65B41DA39758}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="2df2684a-2237-489e-8795-1f946593e18f" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="3ddbdfa1-be50-4b7a-b66f-14c4748c8596">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{712A39FB-A1FD-418D-A657-32ECBACC94FF}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -2281,4 +2262,23 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{29D94F07-D8B4-4F0F-9836-65B41DA39758}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1F55CD33-1A0B-42F8-BD7E-0D32351F432C}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="2df2684a-2237-489e-8795-1f946593e18f"/>
+    <ds:schemaRef ds:uri="3ddbdfa1-be50-4b7a-b66f-14c4748c8596"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
update settlement info; bump version to 0.3.4
</commit_message>
<xml_diff>
--- a/data/settlement info/settlement info.xlsx
+++ b/data/settlement info/settlement info.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://hp.sharepoint.com/teams/InputDevice/Shared Documents/General/17. Automation Projects/settlement-form-generator/data/settlement info/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="28" documentId="13_ncr:1_{EFC9C18D-6AB1-419E-98A5-91AC95941D19}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1858AAC7-D250-40AF-91D2-BC06E6EAAEF8}"/>
+  <xr:revisionPtr revIDLastSave="29" documentId="13_ncr:1_{EFC9C18D-6AB1-419E-98A5-91AC95941D19}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1F6DA322-6E2C-4C44-B731-6DDB2D6806DF}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{B4B4C7C1-7052-47F5-B23D-E78807A6AB18}"/>
   </bookViews>
@@ -365,9 +365,6 @@
     <t>Sunrex</t>
   </si>
   <si>
-    <t>SUNREX TECHNOLOGY CORP.</t>
-  </si>
-  <si>
     <t>Ellie Chen</t>
   </si>
   <si>
@@ -572,6 +569,9 @@
   </si>
   <si>
     <t>SR_000025</t>
+  </si>
+  <si>
+    <t>SUNREX TECHNOLOGY CORP</t>
   </si>
 </sst>
 </file>
@@ -1033,37 +1033,37 @@
   <sheetData>
     <row r="1" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="C1" s="1" t="s">
+        <v>126</v>
+      </c>
+      <c r="D1" s="1" t="s">
         <v>127</v>
       </c>
-      <c r="D1" s="1" t="s">
-        <v>128</v>
-      </c>
       <c r="E1" s="1" t="s">
+        <v>122</v>
+      </c>
+      <c r="F1" s="1" t="s">
         <v>123</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="G1" s="1" t="s">
+        <v>125</v>
+      </c>
+      <c r="H1" s="1" t="s">
         <v>124</v>
       </c>
-      <c r="G1" s="1" t="s">
-        <v>126</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>125</v>
-      </c>
       <c r="I1" s="1" t="s">
+        <v>129</v>
+      </c>
+      <c r="J1" s="1" t="s">
         <v>130</v>
       </c>
-      <c r="J1" s="1" t="s">
-        <v>131</v>
-      </c>
       <c r="K1" s="1" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
     </row>
     <row r="2" spans="1:11" ht="16.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -1080,22 +1080,22 @@
         <v>4</v>
       </c>
       <c r="F2" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="G2" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="H2" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="I2" s="2">
         <v>45727</v>
       </c>
       <c r="J2" s="2" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="K2" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
     </row>
     <row r="3" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.35">
@@ -1115,19 +1115,19 @@
         <v>9</v>
       </c>
       <c r="G3" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="H3" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="I3" s="2">
         <v>45722</v>
       </c>
       <c r="J3" s="2" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="K3" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
     </row>
     <row r="4" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.35">
@@ -1147,16 +1147,16 @@
         <v>5</v>
       </c>
       <c r="G4" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="H4" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="I4" s="2">
         <v>45785</v>
       </c>
       <c r="J4" s="2" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
     </row>
     <row r="5" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.35">
@@ -1176,19 +1176,19 @@
         <v>16</v>
       </c>
       <c r="G5" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="H5" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="I5" s="2">
         <v>45784</v>
       </c>
       <c r="J5" s="2" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="K5" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
     </row>
     <row r="6" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.35">
@@ -1208,19 +1208,19 @@
         <v>20</v>
       </c>
       <c r="G6" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="H6" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="I6" s="2">
         <v>45729</v>
       </c>
       <c r="J6" s="2" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="K6" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
     </row>
     <row r="7" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.35">
@@ -1240,19 +1240,19 @@
         <v>24</v>
       </c>
       <c r="G7" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="H7" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="I7" s="2">
         <v>45924</v>
       </c>
       <c r="J7" s="2" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="K7" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
     </row>
     <row r="8" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.35">
@@ -1272,19 +1272,19 @@
         <v>5</v>
       </c>
       <c r="G8" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="H8" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="I8" s="2">
         <v>45729</v>
       </c>
       <c r="J8" s="2" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="K8" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
     </row>
     <row r="9" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.35">
@@ -1304,19 +1304,19 @@
         <v>5</v>
       </c>
       <c r="G9" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="H9" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="I9" s="2">
         <v>45722</v>
       </c>
       <c r="J9" s="2" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="K9" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
     </row>
     <row r="10" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.35">
@@ -1336,19 +1336,19 @@
         <v>5</v>
       </c>
       <c r="G10" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="H10" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="I10" s="2">
         <v>45740</v>
       </c>
       <c r="J10" s="2" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="K10" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
     </row>
     <row r="11" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.35">
@@ -1368,19 +1368,19 @@
         <v>5</v>
       </c>
       <c r="G11" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="H11" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="I11" s="2">
         <v>45723</v>
       </c>
       <c r="J11" s="2" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="K11" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
     </row>
     <row r="12" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.35">
@@ -1400,16 +1400,16 @@
         <v>40</v>
       </c>
       <c r="G12" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="H12" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="I12" s="2">
         <v>45722</v>
       </c>
       <c r="J12" s="2" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
     </row>
     <row r="13" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.35">
@@ -1429,14 +1429,14 @@
         <v>45</v>
       </c>
       <c r="G13" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="H13" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="I13" s="2"/>
       <c r="J13" s="2" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
     </row>
     <row r="14" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.35">
@@ -1456,16 +1456,16 @@
         <v>49</v>
       </c>
       <c r="G14" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="H14" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="I14" s="2">
         <v>45791</v>
       </c>
       <c r="J14" s="2" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
     </row>
     <row r="15" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.35">
@@ -1485,19 +1485,19 @@
         <v>54</v>
       </c>
       <c r="G15" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="H15" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="I15" s="2">
         <v>45740</v>
       </c>
       <c r="J15" s="2" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="K15" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
     </row>
     <row r="16" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.35">
@@ -1517,16 +1517,16 @@
         <v>58</v>
       </c>
       <c r="G16" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="H16" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="I16" s="2">
         <v>45784</v>
       </c>
       <c r="J16" s="2" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
     </row>
     <row r="17" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.35">
@@ -1546,19 +1546,19 @@
         <v>63</v>
       </c>
       <c r="G17" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="H17" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="I17" s="2">
         <v>45740</v>
       </c>
       <c r="J17" s="2" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="K17" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
     </row>
     <row r="18" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.35">
@@ -1578,17 +1578,17 @@
         <v>67</v>
       </c>
       <c r="G18" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="H18" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="I18" s="2"/>
       <c r="J18" s="2" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="K18" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
     </row>
     <row r="19" spans="1:11" ht="16.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -1608,17 +1608,17 @@
         <v>45</v>
       </c>
       <c r="G19" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="H19" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="I19" s="2"/>
       <c r="J19" s="2" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="K19" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
     </row>
     <row r="20" spans="1:11" ht="16.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -1638,19 +1638,19 @@
         <v>74</v>
       </c>
       <c r="G20" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="H20" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="I20" s="2">
         <v>45798</v>
       </c>
       <c r="J20" s="2" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="K20" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
     </row>
     <row r="21" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.35">
@@ -1670,10 +1670,10 @@
         <v>78</v>
       </c>
       <c r="G21" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="H21" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="I21" s="2"/>
       <c r="J21" s="2"/>
@@ -1695,14 +1695,14 @@
         <v>78</v>
       </c>
       <c r="G22" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="H22" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="I22" s="2"/>
       <c r="J22" s="2" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
     </row>
     <row r="23" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.35">
@@ -1722,14 +1722,14 @@
         <v>85</v>
       </c>
       <c r="G23" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="H23" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="I23" s="2"/>
       <c r="J23" s="2" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
     </row>
     <row r="24" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.35">
@@ -1752,16 +1752,16 @@
         <v>91</v>
       </c>
       <c r="G24" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="H24" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="I24" s="2">
         <v>45666</v>
       </c>
       <c r="J24" s="2" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="K24" t="s">
         <v>92</v>
@@ -1787,16 +1787,16 @@
         <v>95</v>
       </c>
       <c r="G25" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="H25" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="I25" s="2">
         <v>45666</v>
       </c>
       <c r="J25" s="2" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="K25" t="s">
         <v>92</v>
@@ -1813,22 +1813,22 @@
         <v>97</v>
       </c>
       <c r="E26" t="s">
+        <v>131</v>
+      </c>
+      <c r="F26" t="s">
         <v>132</v>
       </c>
-      <c r="F26" t="s">
-        <v>133</v>
-      </c>
       <c r="G26" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="H26" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="I26" s="2">
         <v>45670</v>
       </c>
       <c r="J26" s="2" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="K26" t="s">
         <v>98</v>
@@ -1851,16 +1851,16 @@
         <v>102</v>
       </c>
       <c r="G27" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="H27" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="I27" s="2">
         <v>45693</v>
       </c>
       <c r="J27" s="2" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="K27" t="s">
         <v>103</v>
@@ -1883,19 +1883,19 @@
         <v>78</v>
       </c>
       <c r="G28" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="H28" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="I28" s="2">
         <v>45666</v>
       </c>
       <c r="J28" s="2" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="K28" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
     </row>
     <row r="29" spans="1:11" ht="16.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -1906,84 +1906,84 @@
         <v>107</v>
       </c>
       <c r="D29" t="s">
+        <v>176</v>
+      </c>
+      <c r="E29" t="s">
         <v>108</v>
-      </c>
-      <c r="E29" t="s">
-        <v>109</v>
       </c>
       <c r="F29" t="s">
         <v>63</v>
       </c>
       <c r="G29" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="H29" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="I29" s="2">
         <v>45672</v>
       </c>
       <c r="J29" s="2" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="K29" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
     </row>
     <row r="30" spans="1:11" ht="16.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
+        <v>110</v>
+      </c>
+      <c r="C30" t="s">
         <v>111</v>
       </c>
-      <c r="C30" t="s">
+      <c r="D30" t="s">
         <v>112</v>
       </c>
-      <c r="D30" t="s">
+      <c r="E30" t="s">
         <v>113</v>
       </c>
-      <c r="E30" t="s">
+      <c r="F30" t="s">
         <v>114</v>
       </c>
-      <c r="F30" t="s">
-        <v>115</v>
-      </c>
       <c r="G30" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="H30" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="I30" s="2">
         <v>45714</v>
       </c>
       <c r="J30" s="2" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
     </row>
     <row r="31" spans="1:11" ht="16.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="C31" t="s">
+        <v>115</v>
+      </c>
+      <c r="D31" t="s">
         <v>116</v>
       </c>
-      <c r="D31" t="s">
+      <c r="E31" t="s">
         <v>117</v>
-      </c>
-      <c r="E31" t="s">
-        <v>118</v>
       </c>
       <c r="F31" t="s">
         <v>5</v>
       </c>
       <c r="G31" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="H31" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="I31" s="2"/>
       <c r="J31" s="2" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
     </row>
   </sheetData>
@@ -1997,6 +1997,26 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="2df2684a-2237-489e-8795-1f946593e18f" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="3ddbdfa1-be50-4b7a-b66f-14c4748c8596">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100C7BB62D9C7AC4249BB50D4F119F8FF50" ma:contentTypeVersion="14" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="dab14850594d04436880d3464ba468af">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="3ddbdfa1-be50-4b7a-b66f-14c4748c8596" xmlns:ns3="2df2684a-2237-489e-8795-1f946593e18f" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="eb8d2f689c1774a9065a5e99593f72e7" ns2:_="" ns3:_="">
     <xsd:import namespace="3ddbdfa1-be50-4b7a-b66f-14c4748c8596"/>
@@ -2225,27 +2245,26 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1F55CD33-1A0B-42F8-BD7E-0D32351F432C}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="2df2684a-2237-489e-8795-1f946593e18f"/>
+    <ds:schemaRef ds:uri="3ddbdfa1-be50-4b7a-b66f-14c4748c8596"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="2df2684a-2237-489e-8795-1f946593e18f" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="3ddbdfa1-be50-4b7a-b66f-14c4748c8596">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{29D94F07-D8B4-4F0F-9836-65B41DA39758}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{712A39FB-A1FD-418D-A657-32ECBACC94FF}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -2262,23 +2281,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{29D94F07-D8B4-4F0F-9836-65B41DA39758}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1F55CD33-1A0B-42F8-BD7E-0D32351F432C}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="2df2684a-2237-489e-8795-1f946593e18f"/>
-    <ds:schemaRef ds:uri="3ddbdfa1-be50-4b7a-b66f-14c4748c8596"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>